<commit_message>
B: correct Excel table headers and complete filter ranges
</commit_message>
<xml_diff>
--- a/docs/data_dictionary_v1.xlsx
+++ b/docs/data_dictionary_v1.xlsx
@@ -164,16 +164,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FieldsTable" displayName="FieldsTable" ref="A5:G343" headerRowCount="1">
-  <autoFilter ref="A5:G343"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="FieldsTable" displayName="FieldsTable" ref="A5:H344" headerRowCount="1">
+  <autoFilter ref="A5:H344"/>
+  <tableColumns count="8">
     <tableColumn id="1" name="Object"/>
     <tableColumn id="2" name="Column"/>
     <tableColumn id="3" name="Type"/>
     <tableColumn id="4" name="PK/FK/uniqueness"/>
     <tableColumn id="5" name="Nullable"/>
     <tableColumn id="6" name="Meaning"/>
-    <tableColumn id="7" name="Status"/>
+    <tableColumn id="7" name="Owner"/>
+    <tableColumn id="8" name="Default"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -185,7 +186,7 @@
   <tableColumns count="4">
     <tableColumn id="1" name="Object"/>
     <tableColumn id="2" name="One row represents"/>
-    <tableColumn id="3" name="Definition status"/>
+    <tableColumn id="3" name="Owner"/>
     <tableColumn id="4" name="Columns"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>

</xml_diff>